<commit_message>
BIS-2697: fixed excel export
</commit_message>
<xml_diff>
--- a/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-data-set-plain-text.xlsx
+++ b/server-application-server/sourceTest/java/ch/ethz/sis/openbis/generic/server/xls/export/resources/export-data-set-plain-text.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="51">
   <si>
     <t xml:space="preserve">DATASET</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t xml:space="preserve">Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meta Data</t>
   </si>
   <si>
     <t xml:space="preserve">Name</t>
@@ -184,7 +187,7 @@
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -224,6 +227,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="13"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -273,7 +284,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -298,11 +309,15 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -314,7 +329,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -335,19 +350,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMX12"/>
-  <sheetFormatPr defaultColWidth="10.5234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:V12"/>
+  <sheetFormatPr defaultColWidth="10.53125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="20.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="7" style="1" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="16.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1035" min="1035" style="1" width="8.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="15" style="1" width="16.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -425,126 +439,128 @@
       <c r="O4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="P4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="R4" s="1"/>
-      <c r="T4" s="1"/>
+      <c r="R4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="S4" s="1"/>
       <c r="U4" s="1"/>
-      <c r="AMV4" s="1"/>
+      <c r="V4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="B5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="C5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="6" t="s">
+      <c r="E5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="F5" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="H5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="6"/>
+      <c r="I5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="7"/>
       <c r="K5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="8" t="s">
         <v>28</v>
       </c>
+      <c r="L5" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="M5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="N5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="O5" s="8" t="s">
+      <c r="N5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="O5" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="P5" s="9"/>
+      <c r="Q5" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="R5" s="1"/>
-      <c r="T5" s="1"/>
+      <c r="R5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="S5" s="1"/>
       <c r="U5" s="1"/>
-      <c r="AMV5" s="1"/>
+      <c r="V5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="B6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="C6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="6" t="s">
+      <c r="E6" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" s="6" t="s">
+      <c r="F6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="J6" s="6"/>
+      <c r="I6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="7"/>
       <c r="K6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="8" t="s">
         <v>28</v>
       </c>
+      <c r="L6" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="M6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="N6" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="O6" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="P6" s="9" t="s">
+      <c r="N6" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="O6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="P6" s="9"/>
+      <c r="Q6" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="R6" s="1"/>
-      <c r="T6" s="1"/>
+      <c r="R6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="S6" s="1"/>
       <c r="U6" s="1"/>
-      <c r="AMV6" s="1"/>
+      <c r="V6" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
@@ -569,13 +585,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" s="9" customFormat="true" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="10" customFormat="true" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>3</v>
       </c>
@@ -621,67 +637,68 @@
       <c r="O11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="5" t="s">
+      <c r="P11" s="6" t="s">
         <v>18</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="AMW11" s="1"/>
-      <c r="AMX11" s="1"/>
+        <v>19</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="7"/>
-      <c r="H12" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="I12" s="6"/>
-      <c r="J12" s="10" t="s">
+      <c r="B12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="8"/>
+      <c r="H12" s="7" t="s">
         <v>46</v>
       </c>
+      <c r="I12" s="7"/>
+      <c r="J12" s="11" t="s">
+        <v>47</v>
+      </c>
       <c r="K12" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="8" t="s">
         <v>28</v>
       </c>
+      <c r="L12" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="M12" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="N12" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="O12" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="P12" s="9" t="s">
+      <c r="N12" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="O12" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="Q12" s="11" t="s">
+      <c r="P12" s="9"/>
+      <c r="Q12" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="R12" s="1"/>
-      <c r="T12" s="1"/>
+      <c r="R12" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="S12" s="1"/>
       <c r="U12" s="1"/>
-      <c r="AMV12" s="1"/>
+      <c r="V12" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>